<commit_message>
fix: remove depreciation columns from Equipment Inventory spreadsheet
User can't know depreciation values at entry time. Removed Depreciation Life,
Annual Depreciation, and Current Book Value columns. Now 11 clean columns.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TotalGuard_2026_Equipment_Inventory.xlsx
+++ b/TotalGuard_2026_Equipment_Inventory.xlsx
@@ -543,7 +543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N103"/>
+  <dimension ref="A1:K103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -556,10 +556,7 @@
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -578,9 +575,6 @@
       <c r="I1" s="2" t="n"/>
       <c r="J1" s="2" t="n"/>
       <c r="K1" s="2" t="n"/>
-      <c r="L1" s="2" t="n"/>
-      <c r="M1" s="2" t="n"/>
-      <c r="N1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -630,25 +624,10 @@
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>Depreciation Life (Yrs)</t>
-        </is>
-      </c>
-      <c r="K2" s="3" t="inlineStr">
-        <is>
-          <t>Annual Depreciation</t>
-        </is>
-      </c>
-      <c r="L2" s="3" t="inlineStr">
-        <is>
-          <t>Current Book Value</t>
-        </is>
-      </c>
-      <c r="M2" s="3" t="inlineStr">
-        <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="N2" s="3" t="inlineStr">
+      <c r="K2" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -684,23 +663,12 @@
         </is>
       </c>
       <c r="I3" s="6" t="inlineStr"/>
-      <c r="J3" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="K3" s="7">
-        <f>IF(J3&gt;0,G3/J3,0)</f>
-        <v/>
-      </c>
-      <c r="L3" s="7">
-        <f>MAX(G3-K3*(YEAR(TODAY())-YEAR(F3)),0)</f>
-        <v/>
-      </c>
-      <c r="M3" s="5" t="inlineStr">
+      <c r="J3" s="5" t="inlineStr">
         <is>
           <t>Truck</t>
         </is>
       </c>
-      <c r="N3" s="5" t="inlineStr"/>
+      <c r="K3" s="5" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="8" t="n">
@@ -732,23 +700,12 @@
         </is>
       </c>
       <c r="I4" s="10" t="inlineStr"/>
-      <c r="J4" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="K4" s="11">
-        <f>IF(J4&gt;0,G4/J4,0)</f>
-        <v/>
-      </c>
-      <c r="L4" s="11">
-        <f>MAX(G4-K4*(YEAR(TODAY())-YEAR(F4)),0)</f>
-        <v/>
-      </c>
-      <c r="M4" s="9" t="inlineStr">
+      <c r="J4" s="9" t="inlineStr">
         <is>
           <t>Office</t>
         </is>
       </c>
-      <c r="N4" s="9" t="inlineStr"/>
+      <c r="K4" s="9" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
@@ -780,23 +737,12 @@
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr"/>
-      <c r="J5" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="K5" s="7">
-        <f>IF(J5&gt;0,G5/J5,0)</f>
-        <v/>
-      </c>
-      <c r="L5" s="7">
-        <f>MAX(G5-K5*(YEAR(TODAY())-YEAR(F5)),0)</f>
-        <v/>
-      </c>
-      <c r="M5" s="5" t="inlineStr">
+      <c r="J5" s="5" t="inlineStr">
         <is>
           <t>Truck</t>
         </is>
       </c>
-      <c r="N5" s="5" t="inlineStr"/>
+      <c r="K5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="8" t="n">
@@ -828,19 +774,8 @@
         </is>
       </c>
       <c r="I6" s="10" t="inlineStr"/>
-      <c r="J6" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="K6" s="11">
-        <f>IF(J6&gt;0,G6/J6,0)</f>
-        <v/>
-      </c>
-      <c r="L6" s="11">
-        <f>MAX(G6-K6*(YEAR(TODAY())-YEAR(F6)),0)</f>
-        <v/>
-      </c>
-      <c r="M6" s="9" t="inlineStr"/>
-      <c r="N6" s="9" t="inlineStr">
+      <c r="J6" s="9" t="inlineStr"/>
+      <c r="K6" s="9" t="inlineStr">
         <is>
           <t>Marketing materials</t>
         </is>
@@ -859,16 +794,7 @@
       <c r="H7" s="5" t="n"/>
       <c r="I7" s="6" t="n"/>
       <c r="J7" s="5" t="n"/>
-      <c r="K7" s="7">
-        <f>IF(J7&gt;0,G7/J7,0)</f>
-        <v/>
-      </c>
-      <c r="L7" s="7">
-        <f>MAX(G7-K7*(YEAR(TODAY())-YEAR(F7)),0)</f>
-        <v/>
-      </c>
-      <c r="M7" s="5" t="n"/>
-      <c r="N7" s="5" t="n"/>
+      <c r="K7" s="5" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="8" t="n">
@@ -883,16 +809,7 @@
       <c r="H8" s="9" t="n"/>
       <c r="I8" s="10" t="n"/>
       <c r="J8" s="9" t="n"/>
-      <c r="K8" s="11">
-        <f>IF(J8&gt;0,G8/J8,0)</f>
-        <v/>
-      </c>
-      <c r="L8" s="11">
-        <f>MAX(G8-K8*(YEAR(TODAY())-YEAR(F8)),0)</f>
-        <v/>
-      </c>
-      <c r="M8" s="9" t="n"/>
-      <c r="N8" s="9" t="n"/>
+      <c r="K8" s="9" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
@@ -907,16 +824,7 @@
       <c r="H9" s="5" t="n"/>
       <c r="I9" s="6" t="n"/>
       <c r="J9" s="5" t="n"/>
-      <c r="K9" s="7">
-        <f>IF(J9&gt;0,G9/J9,0)</f>
-        <v/>
-      </c>
-      <c r="L9" s="7">
-        <f>MAX(G9-K9*(YEAR(TODAY())-YEAR(F9)),0)</f>
-        <v/>
-      </c>
-      <c r="M9" s="5" t="n"/>
-      <c r="N9" s="5" t="n"/>
+      <c r="K9" s="5" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="8" t="n">
@@ -931,16 +839,7 @@
       <c r="H10" s="9" t="n"/>
       <c r="I10" s="10" t="n"/>
       <c r="J10" s="9" t="n"/>
-      <c r="K10" s="11">
-        <f>IF(J10&gt;0,G10/J10,0)</f>
-        <v/>
-      </c>
-      <c r="L10" s="11">
-        <f>MAX(G10-K10*(YEAR(TODAY())-YEAR(F10)),0)</f>
-        <v/>
-      </c>
-      <c r="M10" s="9" t="n"/>
-      <c r="N10" s="9" t="n"/>
+      <c r="K10" s="9" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
@@ -955,16 +854,7 @@
       <c r="H11" s="5" t="n"/>
       <c r="I11" s="6" t="n"/>
       <c r="J11" s="5" t="n"/>
-      <c r="K11" s="7">
-        <f>IF(J11&gt;0,G11/J11,0)</f>
-        <v/>
-      </c>
-      <c r="L11" s="7">
-        <f>MAX(G11-K11*(YEAR(TODAY())-YEAR(F11)),0)</f>
-        <v/>
-      </c>
-      <c r="M11" s="5" t="n"/>
-      <c r="N11" s="5" t="n"/>
+      <c r="K11" s="5" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="8" t="n">
@@ -979,16 +869,7 @@
       <c r="H12" s="9" t="n"/>
       <c r="I12" s="10" t="n"/>
       <c r="J12" s="9" t="n"/>
-      <c r="K12" s="11">
-        <f>IF(J12&gt;0,G12/J12,0)</f>
-        <v/>
-      </c>
-      <c r="L12" s="11">
-        <f>MAX(G12-K12*(YEAR(TODAY())-YEAR(F12)),0)</f>
-        <v/>
-      </c>
-      <c r="M12" s="9" t="n"/>
-      <c r="N12" s="9" t="n"/>
+      <c r="K12" s="9" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
@@ -1003,16 +884,7 @@
       <c r="H13" s="5" t="n"/>
       <c r="I13" s="6" t="n"/>
       <c r="J13" s="5" t="n"/>
-      <c r="K13" s="7">
-        <f>IF(J13&gt;0,G13/J13,0)</f>
-        <v/>
-      </c>
-      <c r="L13" s="7">
-        <f>MAX(G13-K13*(YEAR(TODAY())-YEAR(F13)),0)</f>
-        <v/>
-      </c>
-      <c r="M13" s="5" t="n"/>
-      <c r="N13" s="5" t="n"/>
+      <c r="K13" s="5" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="8" t="n">
@@ -1027,16 +899,7 @@
       <c r="H14" s="9" t="n"/>
       <c r="I14" s="10" t="n"/>
       <c r="J14" s="9" t="n"/>
-      <c r="K14" s="11">
-        <f>IF(J14&gt;0,G14/J14,0)</f>
-        <v/>
-      </c>
-      <c r="L14" s="11">
-        <f>MAX(G14-K14*(YEAR(TODAY())-YEAR(F14)),0)</f>
-        <v/>
-      </c>
-      <c r="M14" s="9" t="n"/>
-      <c r="N14" s="9" t="n"/>
+      <c r="K14" s="9" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
@@ -1051,16 +914,7 @@
       <c r="H15" s="5" t="n"/>
       <c r="I15" s="6" t="n"/>
       <c r="J15" s="5" t="n"/>
-      <c r="K15" s="7">
-        <f>IF(J15&gt;0,G15/J15,0)</f>
-        <v/>
-      </c>
-      <c r="L15" s="7">
-        <f>MAX(G15-K15*(YEAR(TODAY())-YEAR(F15)),0)</f>
-        <v/>
-      </c>
-      <c r="M15" s="5" t="n"/>
-      <c r="N15" s="5" t="n"/>
+      <c r="K15" s="5" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="8" t="n">
@@ -1075,16 +929,7 @@
       <c r="H16" s="9" t="n"/>
       <c r="I16" s="10" t="n"/>
       <c r="J16" s="9" t="n"/>
-      <c r="K16" s="11">
-        <f>IF(J16&gt;0,G16/J16,0)</f>
-        <v/>
-      </c>
-      <c r="L16" s="11">
-        <f>MAX(G16-K16*(YEAR(TODAY())-YEAR(F16)),0)</f>
-        <v/>
-      </c>
-      <c r="M16" s="9" t="n"/>
-      <c r="N16" s="9" t="n"/>
+      <c r="K16" s="9" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
@@ -1099,16 +944,7 @@
       <c r="H17" s="5" t="n"/>
       <c r="I17" s="6" t="n"/>
       <c r="J17" s="5" t="n"/>
-      <c r="K17" s="7">
-        <f>IF(J17&gt;0,G17/J17,0)</f>
-        <v/>
-      </c>
-      <c r="L17" s="7">
-        <f>MAX(G17-K17*(YEAR(TODAY())-YEAR(F17)),0)</f>
-        <v/>
-      </c>
-      <c r="M17" s="5" t="n"/>
-      <c r="N17" s="5" t="n"/>
+      <c r="K17" s="5" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="8" t="n">
@@ -1123,16 +959,7 @@
       <c r="H18" s="9" t="n"/>
       <c r="I18" s="10" t="n"/>
       <c r="J18" s="9" t="n"/>
-      <c r="K18" s="11">
-        <f>IF(J18&gt;0,G18/J18,0)</f>
-        <v/>
-      </c>
-      <c r="L18" s="11">
-        <f>MAX(G18-K18*(YEAR(TODAY())-YEAR(F18)),0)</f>
-        <v/>
-      </c>
-      <c r="M18" s="9" t="n"/>
-      <c r="N18" s="9" t="n"/>
+      <c r="K18" s="9" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
@@ -1147,16 +974,7 @@
       <c r="H19" s="5" t="n"/>
       <c r="I19" s="6" t="n"/>
       <c r="J19" s="5" t="n"/>
-      <c r="K19" s="7">
-        <f>IF(J19&gt;0,G19/J19,0)</f>
-        <v/>
-      </c>
-      <c r="L19" s="7">
-        <f>MAX(G19-K19*(YEAR(TODAY())-YEAR(F19)),0)</f>
-        <v/>
-      </c>
-      <c r="M19" s="5" t="n"/>
-      <c r="N19" s="5" t="n"/>
+      <c r="K19" s="5" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="8" t="n">
@@ -1171,16 +989,7 @@
       <c r="H20" s="9" t="n"/>
       <c r="I20" s="10" t="n"/>
       <c r="J20" s="9" t="n"/>
-      <c r="K20" s="11">
-        <f>IF(J20&gt;0,G20/J20,0)</f>
-        <v/>
-      </c>
-      <c r="L20" s="11">
-        <f>MAX(G20-K20*(YEAR(TODAY())-YEAR(F20)),0)</f>
-        <v/>
-      </c>
-      <c r="M20" s="9" t="n"/>
-      <c r="N20" s="9" t="n"/>
+      <c r="K20" s="9" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
@@ -1195,16 +1004,7 @@
       <c r="H21" s="5" t="n"/>
       <c r="I21" s="6" t="n"/>
       <c r="J21" s="5" t="n"/>
-      <c r="K21" s="7">
-        <f>IF(J21&gt;0,G21/J21,0)</f>
-        <v/>
-      </c>
-      <c r="L21" s="7">
-        <f>MAX(G21-K21*(YEAR(TODAY())-YEAR(F21)),0)</f>
-        <v/>
-      </c>
-      <c r="M21" s="5" t="n"/>
-      <c r="N21" s="5" t="n"/>
+      <c r="K21" s="5" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="8" t="n">
@@ -1219,16 +1019,7 @@
       <c r="H22" s="9" t="n"/>
       <c r="I22" s="10" t="n"/>
       <c r="J22" s="9" t="n"/>
-      <c r="K22" s="11">
-        <f>IF(J22&gt;0,G22/J22,0)</f>
-        <v/>
-      </c>
-      <c r="L22" s="11">
-        <f>MAX(G22-K22*(YEAR(TODAY())-YEAR(F22)),0)</f>
-        <v/>
-      </c>
-      <c r="M22" s="9" t="n"/>
-      <c r="N22" s="9" t="n"/>
+      <c r="K22" s="9" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
@@ -1243,16 +1034,7 @@
       <c r="H23" s="5" t="n"/>
       <c r="I23" s="6" t="n"/>
       <c r="J23" s="5" t="n"/>
-      <c r="K23" s="7">
-        <f>IF(J23&gt;0,G23/J23,0)</f>
-        <v/>
-      </c>
-      <c r="L23" s="7">
-        <f>MAX(G23-K23*(YEAR(TODAY())-YEAR(F23)),0)</f>
-        <v/>
-      </c>
-      <c r="M23" s="5" t="n"/>
-      <c r="N23" s="5" t="n"/>
+      <c r="K23" s="5" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="8" t="n">
@@ -1267,16 +1049,7 @@
       <c r="H24" s="9" t="n"/>
       <c r="I24" s="10" t="n"/>
       <c r="J24" s="9" t="n"/>
-      <c r="K24" s="11">
-        <f>IF(J24&gt;0,G24/J24,0)</f>
-        <v/>
-      </c>
-      <c r="L24" s="11">
-        <f>MAX(G24-K24*(YEAR(TODAY())-YEAR(F24)),0)</f>
-        <v/>
-      </c>
-      <c r="M24" s="9" t="n"/>
-      <c r="N24" s="9" t="n"/>
+      <c r="K24" s="9" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
@@ -1291,16 +1064,7 @@
       <c r="H25" s="5" t="n"/>
       <c r="I25" s="6" t="n"/>
       <c r="J25" s="5" t="n"/>
-      <c r="K25" s="7">
-        <f>IF(J25&gt;0,G25/J25,0)</f>
-        <v/>
-      </c>
-      <c r="L25" s="7">
-        <f>MAX(G25-K25*(YEAR(TODAY())-YEAR(F25)),0)</f>
-        <v/>
-      </c>
-      <c r="M25" s="5" t="n"/>
-      <c r="N25" s="5" t="n"/>
+      <c r="K25" s="5" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="8" t="n">
@@ -1315,16 +1079,7 @@
       <c r="H26" s="9" t="n"/>
       <c r="I26" s="10" t="n"/>
       <c r="J26" s="9" t="n"/>
-      <c r="K26" s="11">
-        <f>IF(J26&gt;0,G26/J26,0)</f>
-        <v/>
-      </c>
-      <c r="L26" s="11">
-        <f>MAX(G26-K26*(YEAR(TODAY())-YEAR(F26)),0)</f>
-        <v/>
-      </c>
-      <c r="M26" s="9" t="n"/>
-      <c r="N26" s="9" t="n"/>
+      <c r="K26" s="9" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
@@ -1339,16 +1094,7 @@
       <c r="H27" s="5" t="n"/>
       <c r="I27" s="6" t="n"/>
       <c r="J27" s="5" t="n"/>
-      <c r="K27" s="7">
-        <f>IF(J27&gt;0,G27/J27,0)</f>
-        <v/>
-      </c>
-      <c r="L27" s="7">
-        <f>MAX(G27-K27*(YEAR(TODAY())-YEAR(F27)),0)</f>
-        <v/>
-      </c>
-      <c r="M27" s="5" t="n"/>
-      <c r="N27" s="5" t="n"/>
+      <c r="K27" s="5" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="8" t="n">
@@ -1363,16 +1109,7 @@
       <c r="H28" s="9" t="n"/>
       <c r="I28" s="10" t="n"/>
       <c r="J28" s="9" t="n"/>
-      <c r="K28" s="11">
-        <f>IF(J28&gt;0,G28/J28,0)</f>
-        <v/>
-      </c>
-      <c r="L28" s="11">
-        <f>MAX(G28-K28*(YEAR(TODAY())-YEAR(F28)),0)</f>
-        <v/>
-      </c>
-      <c r="M28" s="9" t="n"/>
-      <c r="N28" s="9" t="n"/>
+      <c r="K28" s="9" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
@@ -1387,16 +1124,7 @@
       <c r="H29" s="5" t="n"/>
       <c r="I29" s="6" t="n"/>
       <c r="J29" s="5" t="n"/>
-      <c r="K29" s="7">
-        <f>IF(J29&gt;0,G29/J29,0)</f>
-        <v/>
-      </c>
-      <c r="L29" s="7">
-        <f>MAX(G29-K29*(YEAR(TODAY())-YEAR(F29)),0)</f>
-        <v/>
-      </c>
-      <c r="M29" s="5" t="n"/>
-      <c r="N29" s="5" t="n"/>
+      <c r="K29" s="5" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="8" t="n">
@@ -1411,16 +1139,7 @@
       <c r="H30" s="9" t="n"/>
       <c r="I30" s="10" t="n"/>
       <c r="J30" s="9" t="n"/>
-      <c r="K30" s="11">
-        <f>IF(J30&gt;0,G30/J30,0)</f>
-        <v/>
-      </c>
-      <c r="L30" s="11">
-        <f>MAX(G30-K30*(YEAR(TODAY())-YEAR(F30)),0)</f>
-        <v/>
-      </c>
-      <c r="M30" s="9" t="n"/>
-      <c r="N30" s="9" t="n"/>
+      <c r="K30" s="9" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
@@ -1435,16 +1154,7 @@
       <c r="H31" s="5" t="n"/>
       <c r="I31" s="6" t="n"/>
       <c r="J31" s="5" t="n"/>
-      <c r="K31" s="7">
-        <f>IF(J31&gt;0,G31/J31,0)</f>
-        <v/>
-      </c>
-      <c r="L31" s="7">
-        <f>MAX(G31-K31*(YEAR(TODAY())-YEAR(F31)),0)</f>
-        <v/>
-      </c>
-      <c r="M31" s="5" t="n"/>
-      <c r="N31" s="5" t="n"/>
+      <c r="K31" s="5" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="8" t="n">
@@ -1459,16 +1169,7 @@
       <c r="H32" s="9" t="n"/>
       <c r="I32" s="10" t="n"/>
       <c r="J32" s="9" t="n"/>
-      <c r="K32" s="11">
-        <f>IF(J32&gt;0,G32/J32,0)</f>
-        <v/>
-      </c>
-      <c r="L32" s="11">
-        <f>MAX(G32-K32*(YEAR(TODAY())-YEAR(F32)),0)</f>
-        <v/>
-      </c>
-      <c r="M32" s="9" t="n"/>
-      <c r="N32" s="9" t="n"/>
+      <c r="K32" s="9" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
@@ -1483,16 +1184,7 @@
       <c r="H33" s="5" t="n"/>
       <c r="I33" s="6" t="n"/>
       <c r="J33" s="5" t="n"/>
-      <c r="K33" s="7">
-        <f>IF(J33&gt;0,G33/J33,0)</f>
-        <v/>
-      </c>
-      <c r="L33" s="7">
-        <f>MAX(G33-K33*(YEAR(TODAY())-YEAR(F33)),0)</f>
-        <v/>
-      </c>
-      <c r="M33" s="5" t="n"/>
-      <c r="N33" s="5" t="n"/>
+      <c r="K33" s="5" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="8" t="n">
@@ -1507,16 +1199,7 @@
       <c r="H34" s="9" t="n"/>
       <c r="I34" s="10" t="n"/>
       <c r="J34" s="9" t="n"/>
-      <c r="K34" s="11">
-        <f>IF(J34&gt;0,G34/J34,0)</f>
-        <v/>
-      </c>
-      <c r="L34" s="11">
-        <f>MAX(G34-K34*(YEAR(TODAY())-YEAR(F34)),0)</f>
-        <v/>
-      </c>
-      <c r="M34" s="9" t="n"/>
-      <c r="N34" s="9" t="n"/>
+      <c r="K34" s="9" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="n">
@@ -1531,16 +1214,7 @@
       <c r="H35" s="5" t="n"/>
       <c r="I35" s="6" t="n"/>
       <c r="J35" s="5" t="n"/>
-      <c r="K35" s="7">
-        <f>IF(J35&gt;0,G35/J35,0)</f>
-        <v/>
-      </c>
-      <c r="L35" s="7">
-        <f>MAX(G35-K35*(YEAR(TODAY())-YEAR(F35)),0)</f>
-        <v/>
-      </c>
-      <c r="M35" s="5" t="n"/>
-      <c r="N35" s="5" t="n"/>
+      <c r="K35" s="5" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="8" t="n">
@@ -1555,16 +1229,7 @@
       <c r="H36" s="9" t="n"/>
       <c r="I36" s="10" t="n"/>
       <c r="J36" s="9" t="n"/>
-      <c r="K36" s="11">
-        <f>IF(J36&gt;0,G36/J36,0)</f>
-        <v/>
-      </c>
-      <c r="L36" s="11">
-        <f>MAX(G36-K36*(YEAR(TODAY())-YEAR(F36)),0)</f>
-        <v/>
-      </c>
-      <c r="M36" s="9" t="n"/>
-      <c r="N36" s="9" t="n"/>
+      <c r="K36" s="9" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="4" t="n">
@@ -1579,16 +1244,7 @@
       <c r="H37" s="5" t="n"/>
       <c r="I37" s="6" t="n"/>
       <c r="J37" s="5" t="n"/>
-      <c r="K37" s="7">
-        <f>IF(J37&gt;0,G37/J37,0)</f>
-        <v/>
-      </c>
-      <c r="L37" s="7">
-        <f>MAX(G37-K37*(YEAR(TODAY())-YEAR(F37)),0)</f>
-        <v/>
-      </c>
-      <c r="M37" s="5" t="n"/>
-      <c r="N37" s="5" t="n"/>
+      <c r="K37" s="5" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="8" t="n">
@@ -1603,16 +1259,7 @@
       <c r="H38" s="9" t="n"/>
       <c r="I38" s="10" t="n"/>
       <c r="J38" s="9" t="n"/>
-      <c r="K38" s="11">
-        <f>IF(J38&gt;0,G38/J38,0)</f>
-        <v/>
-      </c>
-      <c r="L38" s="11">
-        <f>MAX(G38-K38*(YEAR(TODAY())-YEAR(F38)),0)</f>
-        <v/>
-      </c>
-      <c r="M38" s="9" t="n"/>
-      <c r="N38" s="9" t="n"/>
+      <c r="K38" s="9" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="n">
@@ -1627,16 +1274,7 @@
       <c r="H39" s="5" t="n"/>
       <c r="I39" s="6" t="n"/>
       <c r="J39" s="5" t="n"/>
-      <c r="K39" s="7">
-        <f>IF(J39&gt;0,G39/J39,0)</f>
-        <v/>
-      </c>
-      <c r="L39" s="7">
-        <f>MAX(G39-K39*(YEAR(TODAY())-YEAR(F39)),0)</f>
-        <v/>
-      </c>
-      <c r="M39" s="5" t="n"/>
-      <c r="N39" s="5" t="n"/>
+      <c r="K39" s="5" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="8" t="n">
@@ -1651,16 +1289,7 @@
       <c r="H40" s="9" t="n"/>
       <c r="I40" s="10" t="n"/>
       <c r="J40" s="9" t="n"/>
-      <c r="K40" s="11">
-        <f>IF(J40&gt;0,G40/J40,0)</f>
-        <v/>
-      </c>
-      <c r="L40" s="11">
-        <f>MAX(G40-K40*(YEAR(TODAY())-YEAR(F40)),0)</f>
-        <v/>
-      </c>
-      <c r="M40" s="9" t="n"/>
-      <c r="N40" s="9" t="n"/>
+      <c r="K40" s="9" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="n">
@@ -1675,16 +1304,7 @@
       <c r="H41" s="5" t="n"/>
       <c r="I41" s="6" t="n"/>
       <c r="J41" s="5" t="n"/>
-      <c r="K41" s="7">
-        <f>IF(J41&gt;0,G41/J41,0)</f>
-        <v/>
-      </c>
-      <c r="L41" s="7">
-        <f>MAX(G41-K41*(YEAR(TODAY())-YEAR(F41)),0)</f>
-        <v/>
-      </c>
-      <c r="M41" s="5" t="n"/>
-      <c r="N41" s="5" t="n"/>
+      <c r="K41" s="5" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="8" t="n">
@@ -1699,16 +1319,7 @@
       <c r="H42" s="9" t="n"/>
       <c r="I42" s="10" t="n"/>
       <c r="J42" s="9" t="n"/>
-      <c r="K42" s="11">
-        <f>IF(J42&gt;0,G42/J42,0)</f>
-        <v/>
-      </c>
-      <c r="L42" s="11">
-        <f>MAX(G42-K42*(YEAR(TODAY())-YEAR(F42)),0)</f>
-        <v/>
-      </c>
-      <c r="M42" s="9" t="n"/>
-      <c r="N42" s="9" t="n"/>
+      <c r="K42" s="9" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="n">
@@ -1723,16 +1334,7 @@
       <c r="H43" s="5" t="n"/>
       <c r="I43" s="6" t="n"/>
       <c r="J43" s="5" t="n"/>
-      <c r="K43" s="7">
-        <f>IF(J43&gt;0,G43/J43,0)</f>
-        <v/>
-      </c>
-      <c r="L43" s="7">
-        <f>MAX(G43-K43*(YEAR(TODAY())-YEAR(F43)),0)</f>
-        <v/>
-      </c>
-      <c r="M43" s="5" t="n"/>
-      <c r="N43" s="5" t="n"/>
+      <c r="K43" s="5" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="8" t="n">
@@ -1747,16 +1349,7 @@
       <c r="H44" s="9" t="n"/>
       <c r="I44" s="10" t="n"/>
       <c r="J44" s="9" t="n"/>
-      <c r="K44" s="11">
-        <f>IF(J44&gt;0,G44/J44,0)</f>
-        <v/>
-      </c>
-      <c r="L44" s="11">
-        <f>MAX(G44-K44*(YEAR(TODAY())-YEAR(F44)),0)</f>
-        <v/>
-      </c>
-      <c r="M44" s="9" t="n"/>
-      <c r="N44" s="9" t="n"/>
+      <c r="K44" s="9" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="n">
@@ -1771,16 +1364,7 @@
       <c r="H45" s="5" t="n"/>
       <c r="I45" s="6" t="n"/>
       <c r="J45" s="5" t="n"/>
-      <c r="K45" s="7">
-        <f>IF(J45&gt;0,G45/J45,0)</f>
-        <v/>
-      </c>
-      <c r="L45" s="7">
-        <f>MAX(G45-K45*(YEAR(TODAY())-YEAR(F45)),0)</f>
-        <v/>
-      </c>
-      <c r="M45" s="5" t="n"/>
-      <c r="N45" s="5" t="n"/>
+      <c r="K45" s="5" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="8" t="n">
@@ -1795,16 +1379,7 @@
       <c r="H46" s="9" t="n"/>
       <c r="I46" s="10" t="n"/>
       <c r="J46" s="9" t="n"/>
-      <c r="K46" s="11">
-        <f>IF(J46&gt;0,G46/J46,0)</f>
-        <v/>
-      </c>
-      <c r="L46" s="11">
-        <f>MAX(G46-K46*(YEAR(TODAY())-YEAR(F46)),0)</f>
-        <v/>
-      </c>
-      <c r="M46" s="9" t="n"/>
-      <c r="N46" s="9" t="n"/>
+      <c r="K46" s="9" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="4" t="n">
@@ -1819,16 +1394,7 @@
       <c r="H47" s="5" t="n"/>
       <c r="I47" s="6" t="n"/>
       <c r="J47" s="5" t="n"/>
-      <c r="K47" s="7">
-        <f>IF(J47&gt;0,G47/J47,0)</f>
-        <v/>
-      </c>
-      <c r="L47" s="7">
-        <f>MAX(G47-K47*(YEAR(TODAY())-YEAR(F47)),0)</f>
-        <v/>
-      </c>
-      <c r="M47" s="5" t="n"/>
-      <c r="N47" s="5" t="n"/>
+      <c r="K47" s="5" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="8" t="n">
@@ -1843,16 +1409,7 @@
       <c r="H48" s="9" t="n"/>
       <c r="I48" s="10" t="n"/>
       <c r="J48" s="9" t="n"/>
-      <c r="K48" s="11">
-        <f>IF(J48&gt;0,G48/J48,0)</f>
-        <v/>
-      </c>
-      <c r="L48" s="11">
-        <f>MAX(G48-K48*(YEAR(TODAY())-YEAR(F48)),0)</f>
-        <v/>
-      </c>
-      <c r="M48" s="9" t="n"/>
-      <c r="N48" s="9" t="n"/>
+      <c r="K48" s="9" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="4" t="n">
@@ -1867,16 +1424,7 @@
       <c r="H49" s="5" t="n"/>
       <c r="I49" s="6" t="n"/>
       <c r="J49" s="5" t="n"/>
-      <c r="K49" s="7">
-        <f>IF(J49&gt;0,G49/J49,0)</f>
-        <v/>
-      </c>
-      <c r="L49" s="7">
-        <f>MAX(G49-K49*(YEAR(TODAY())-YEAR(F49)),0)</f>
-        <v/>
-      </c>
-      <c r="M49" s="5" t="n"/>
-      <c r="N49" s="5" t="n"/>
+      <c r="K49" s="5" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="8" t="n">
@@ -1891,16 +1439,7 @@
       <c r="H50" s="9" t="n"/>
       <c r="I50" s="10" t="n"/>
       <c r="J50" s="9" t="n"/>
-      <c r="K50" s="11">
-        <f>IF(J50&gt;0,G50/J50,0)</f>
-        <v/>
-      </c>
-      <c r="L50" s="11">
-        <f>MAX(G50-K50*(YEAR(TODAY())-YEAR(F50)),0)</f>
-        <v/>
-      </c>
-      <c r="M50" s="9" t="n"/>
-      <c r="N50" s="9" t="n"/>
+      <c r="K50" s="9" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="4" t="n">
@@ -1915,16 +1454,7 @@
       <c r="H51" s="5" t="n"/>
       <c r="I51" s="6" t="n"/>
       <c r="J51" s="5" t="n"/>
-      <c r="K51" s="7">
-        <f>IF(J51&gt;0,G51/J51,0)</f>
-        <v/>
-      </c>
-      <c r="L51" s="7">
-        <f>MAX(G51-K51*(YEAR(TODAY())-YEAR(F51)),0)</f>
-        <v/>
-      </c>
-      <c r="M51" s="5" t="n"/>
-      <c r="N51" s="5" t="n"/>
+      <c r="K51" s="5" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="8" t="n">
@@ -1939,16 +1469,7 @@
       <c r="H52" s="9" t="n"/>
       <c r="I52" s="10" t="n"/>
       <c r="J52" s="9" t="n"/>
-      <c r="K52" s="11">
-        <f>IF(J52&gt;0,G52/J52,0)</f>
-        <v/>
-      </c>
-      <c r="L52" s="11">
-        <f>MAX(G52-K52*(YEAR(TODAY())-YEAR(F52)),0)</f>
-        <v/>
-      </c>
-      <c r="M52" s="9" t="n"/>
-      <c r="N52" s="9" t="n"/>
+      <c r="K52" s="9" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="4" t="n">
@@ -1963,16 +1484,7 @@
       <c r="H53" s="5" t="n"/>
       <c r="I53" s="6" t="n"/>
       <c r="J53" s="5" t="n"/>
-      <c r="K53" s="7">
-        <f>IF(J53&gt;0,G53/J53,0)</f>
-        <v/>
-      </c>
-      <c r="L53" s="7">
-        <f>MAX(G53-K53*(YEAR(TODAY())-YEAR(F53)),0)</f>
-        <v/>
-      </c>
-      <c r="M53" s="5" t="n"/>
-      <c r="N53" s="5" t="n"/>
+      <c r="K53" s="5" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="8" t="n">
@@ -1987,16 +1499,7 @@
       <c r="H54" s="9" t="n"/>
       <c r="I54" s="10" t="n"/>
       <c r="J54" s="9" t="n"/>
-      <c r="K54" s="11">
-        <f>IF(J54&gt;0,G54/J54,0)</f>
-        <v/>
-      </c>
-      <c r="L54" s="11">
-        <f>MAX(G54-K54*(YEAR(TODAY())-YEAR(F54)),0)</f>
-        <v/>
-      </c>
-      <c r="M54" s="9" t="n"/>
-      <c r="N54" s="9" t="n"/>
+      <c r="K54" s="9" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="4" t="n">
@@ -2011,16 +1514,7 @@
       <c r="H55" s="5" t="n"/>
       <c r="I55" s="6" t="n"/>
       <c r="J55" s="5" t="n"/>
-      <c r="K55" s="7">
-        <f>IF(J55&gt;0,G55/J55,0)</f>
-        <v/>
-      </c>
-      <c r="L55" s="7">
-        <f>MAX(G55-K55*(YEAR(TODAY())-YEAR(F55)),0)</f>
-        <v/>
-      </c>
-      <c r="M55" s="5" t="n"/>
-      <c r="N55" s="5" t="n"/>
+      <c r="K55" s="5" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="8" t="n">
@@ -2035,16 +1529,7 @@
       <c r="H56" s="9" t="n"/>
       <c r="I56" s="10" t="n"/>
       <c r="J56" s="9" t="n"/>
-      <c r="K56" s="11">
-        <f>IF(J56&gt;0,G56/J56,0)</f>
-        <v/>
-      </c>
-      <c r="L56" s="11">
-        <f>MAX(G56-K56*(YEAR(TODAY())-YEAR(F56)),0)</f>
-        <v/>
-      </c>
-      <c r="M56" s="9" t="n"/>
-      <c r="N56" s="9" t="n"/>
+      <c r="K56" s="9" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="4" t="n">
@@ -2059,16 +1544,7 @@
       <c r="H57" s="5" t="n"/>
       <c r="I57" s="6" t="n"/>
       <c r="J57" s="5" t="n"/>
-      <c r="K57" s="7">
-        <f>IF(J57&gt;0,G57/J57,0)</f>
-        <v/>
-      </c>
-      <c r="L57" s="7">
-        <f>MAX(G57-K57*(YEAR(TODAY())-YEAR(F57)),0)</f>
-        <v/>
-      </c>
-      <c r="M57" s="5" t="n"/>
-      <c r="N57" s="5" t="n"/>
+      <c r="K57" s="5" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="8" t="n">
@@ -2083,16 +1559,7 @@
       <c r="H58" s="9" t="n"/>
       <c r="I58" s="10" t="n"/>
       <c r="J58" s="9" t="n"/>
-      <c r="K58" s="11">
-        <f>IF(J58&gt;0,G58/J58,0)</f>
-        <v/>
-      </c>
-      <c r="L58" s="11">
-        <f>MAX(G58-K58*(YEAR(TODAY())-YEAR(F58)),0)</f>
-        <v/>
-      </c>
-      <c r="M58" s="9" t="n"/>
-      <c r="N58" s="9" t="n"/>
+      <c r="K58" s="9" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="4" t="n">
@@ -2107,16 +1574,7 @@
       <c r="H59" s="5" t="n"/>
       <c r="I59" s="6" t="n"/>
       <c r="J59" s="5" t="n"/>
-      <c r="K59" s="7">
-        <f>IF(J59&gt;0,G59/J59,0)</f>
-        <v/>
-      </c>
-      <c r="L59" s="7">
-        <f>MAX(G59-K59*(YEAR(TODAY())-YEAR(F59)),0)</f>
-        <v/>
-      </c>
-      <c r="M59" s="5" t="n"/>
-      <c r="N59" s="5" t="n"/>
+      <c r="K59" s="5" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="8" t="n">
@@ -2131,16 +1589,7 @@
       <c r="H60" s="9" t="n"/>
       <c r="I60" s="10" t="n"/>
       <c r="J60" s="9" t="n"/>
-      <c r="K60" s="11">
-        <f>IF(J60&gt;0,G60/J60,0)</f>
-        <v/>
-      </c>
-      <c r="L60" s="11">
-        <f>MAX(G60-K60*(YEAR(TODAY())-YEAR(F60)),0)</f>
-        <v/>
-      </c>
-      <c r="M60" s="9" t="n"/>
-      <c r="N60" s="9" t="n"/>
+      <c r="K60" s="9" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="4" t="n">
@@ -2155,16 +1604,7 @@
       <c r="H61" s="5" t="n"/>
       <c r="I61" s="6" t="n"/>
       <c r="J61" s="5" t="n"/>
-      <c r="K61" s="7">
-        <f>IF(J61&gt;0,G61/J61,0)</f>
-        <v/>
-      </c>
-      <c r="L61" s="7">
-        <f>MAX(G61-K61*(YEAR(TODAY())-YEAR(F61)),0)</f>
-        <v/>
-      </c>
-      <c r="M61" s="5" t="n"/>
-      <c r="N61" s="5" t="n"/>
+      <c r="K61" s="5" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="8" t="n">
@@ -2179,16 +1619,7 @@
       <c r="H62" s="9" t="n"/>
       <c r="I62" s="10" t="n"/>
       <c r="J62" s="9" t="n"/>
-      <c r="K62" s="11">
-        <f>IF(J62&gt;0,G62/J62,0)</f>
-        <v/>
-      </c>
-      <c r="L62" s="11">
-        <f>MAX(G62-K62*(YEAR(TODAY())-YEAR(F62)),0)</f>
-        <v/>
-      </c>
-      <c r="M62" s="9" t="n"/>
-      <c r="N62" s="9" t="n"/>
+      <c r="K62" s="9" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="4" t="n">
@@ -2203,16 +1634,7 @@
       <c r="H63" s="5" t="n"/>
       <c r="I63" s="6" t="n"/>
       <c r="J63" s="5" t="n"/>
-      <c r="K63" s="7">
-        <f>IF(J63&gt;0,G63/J63,0)</f>
-        <v/>
-      </c>
-      <c r="L63" s="7">
-        <f>MAX(G63-K63*(YEAR(TODAY())-YEAR(F63)),0)</f>
-        <v/>
-      </c>
-      <c r="M63" s="5" t="n"/>
-      <c r="N63" s="5" t="n"/>
+      <c r="K63" s="5" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="8" t="n">
@@ -2227,16 +1649,7 @@
       <c r="H64" s="9" t="n"/>
       <c r="I64" s="10" t="n"/>
       <c r="J64" s="9" t="n"/>
-      <c r="K64" s="11">
-        <f>IF(J64&gt;0,G64/J64,0)</f>
-        <v/>
-      </c>
-      <c r="L64" s="11">
-        <f>MAX(G64-K64*(YEAR(TODAY())-YEAR(F64)),0)</f>
-        <v/>
-      </c>
-      <c r="M64" s="9" t="n"/>
-      <c r="N64" s="9" t="n"/>
+      <c r="K64" s="9" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="4" t="n">
@@ -2251,16 +1664,7 @@
       <c r="H65" s="5" t="n"/>
       <c r="I65" s="6" t="n"/>
       <c r="J65" s="5" t="n"/>
-      <c r="K65" s="7">
-        <f>IF(J65&gt;0,G65/J65,0)</f>
-        <v/>
-      </c>
-      <c r="L65" s="7">
-        <f>MAX(G65-K65*(YEAR(TODAY())-YEAR(F65)),0)</f>
-        <v/>
-      </c>
-      <c r="M65" s="5" t="n"/>
-      <c r="N65" s="5" t="n"/>
+      <c r="K65" s="5" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="8" t="n">
@@ -2275,16 +1679,7 @@
       <c r="H66" s="9" t="n"/>
       <c r="I66" s="10" t="n"/>
       <c r="J66" s="9" t="n"/>
-      <c r="K66" s="11">
-        <f>IF(J66&gt;0,G66/J66,0)</f>
-        <v/>
-      </c>
-      <c r="L66" s="11">
-        <f>MAX(G66-K66*(YEAR(TODAY())-YEAR(F66)),0)</f>
-        <v/>
-      </c>
-      <c r="M66" s="9" t="n"/>
-      <c r="N66" s="9" t="n"/>
+      <c r="K66" s="9" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="4" t="n">
@@ -2299,16 +1694,7 @@
       <c r="H67" s="5" t="n"/>
       <c r="I67" s="6" t="n"/>
       <c r="J67" s="5" t="n"/>
-      <c r="K67" s="7">
-        <f>IF(J67&gt;0,G67/J67,0)</f>
-        <v/>
-      </c>
-      <c r="L67" s="7">
-        <f>MAX(G67-K67*(YEAR(TODAY())-YEAR(F67)),0)</f>
-        <v/>
-      </c>
-      <c r="M67" s="5" t="n"/>
-      <c r="N67" s="5" t="n"/>
+      <c r="K67" s="5" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="8" t="n">
@@ -2323,16 +1709,7 @@
       <c r="H68" s="9" t="n"/>
       <c r="I68" s="10" t="n"/>
       <c r="J68" s="9" t="n"/>
-      <c r="K68" s="11">
-        <f>IF(J68&gt;0,G68/J68,0)</f>
-        <v/>
-      </c>
-      <c r="L68" s="11">
-        <f>MAX(G68-K68*(YEAR(TODAY())-YEAR(F68)),0)</f>
-        <v/>
-      </c>
-      <c r="M68" s="9" t="n"/>
-      <c r="N68" s="9" t="n"/>
+      <c r="K68" s="9" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="4" t="n">
@@ -2347,16 +1724,7 @@
       <c r="H69" s="5" t="n"/>
       <c r="I69" s="6" t="n"/>
       <c r="J69" s="5" t="n"/>
-      <c r="K69" s="7">
-        <f>IF(J69&gt;0,G69/J69,0)</f>
-        <v/>
-      </c>
-      <c r="L69" s="7">
-        <f>MAX(G69-K69*(YEAR(TODAY())-YEAR(F69)),0)</f>
-        <v/>
-      </c>
-      <c r="M69" s="5" t="n"/>
-      <c r="N69" s="5" t="n"/>
+      <c r="K69" s="5" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="8" t="n">
@@ -2371,16 +1739,7 @@
       <c r="H70" s="9" t="n"/>
       <c r="I70" s="10" t="n"/>
       <c r="J70" s="9" t="n"/>
-      <c r="K70" s="11">
-        <f>IF(J70&gt;0,G70/J70,0)</f>
-        <v/>
-      </c>
-      <c r="L70" s="11">
-        <f>MAX(G70-K70*(YEAR(TODAY())-YEAR(F70)),0)</f>
-        <v/>
-      </c>
-      <c r="M70" s="9" t="n"/>
-      <c r="N70" s="9" t="n"/>
+      <c r="K70" s="9" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="4" t="n">
@@ -2395,16 +1754,7 @@
       <c r="H71" s="5" t="n"/>
       <c r="I71" s="6" t="n"/>
       <c r="J71" s="5" t="n"/>
-      <c r="K71" s="7">
-        <f>IF(J71&gt;0,G71/J71,0)</f>
-        <v/>
-      </c>
-      <c r="L71" s="7">
-        <f>MAX(G71-K71*(YEAR(TODAY())-YEAR(F71)),0)</f>
-        <v/>
-      </c>
-      <c r="M71" s="5" t="n"/>
-      <c r="N71" s="5" t="n"/>
+      <c r="K71" s="5" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="8" t="n">
@@ -2419,16 +1769,7 @@
       <c r="H72" s="9" t="n"/>
       <c r="I72" s="10" t="n"/>
       <c r="J72" s="9" t="n"/>
-      <c r="K72" s="11">
-        <f>IF(J72&gt;0,G72/J72,0)</f>
-        <v/>
-      </c>
-      <c r="L72" s="11">
-        <f>MAX(G72-K72*(YEAR(TODAY())-YEAR(F72)),0)</f>
-        <v/>
-      </c>
-      <c r="M72" s="9" t="n"/>
-      <c r="N72" s="9" t="n"/>
+      <c r="K72" s="9" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="4" t="n">
@@ -2443,16 +1784,7 @@
       <c r="H73" s="5" t="n"/>
       <c r="I73" s="6" t="n"/>
       <c r="J73" s="5" t="n"/>
-      <c r="K73" s="7">
-        <f>IF(J73&gt;0,G73/J73,0)</f>
-        <v/>
-      </c>
-      <c r="L73" s="7">
-        <f>MAX(G73-K73*(YEAR(TODAY())-YEAR(F73)),0)</f>
-        <v/>
-      </c>
-      <c r="M73" s="5" t="n"/>
-      <c r="N73" s="5" t="n"/>
+      <c r="K73" s="5" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="8" t="n">
@@ -2467,16 +1799,7 @@
       <c r="H74" s="9" t="n"/>
       <c r="I74" s="10" t="n"/>
       <c r="J74" s="9" t="n"/>
-      <c r="K74" s="11">
-        <f>IF(J74&gt;0,G74/J74,0)</f>
-        <v/>
-      </c>
-      <c r="L74" s="11">
-        <f>MAX(G74-K74*(YEAR(TODAY())-YEAR(F74)),0)</f>
-        <v/>
-      </c>
-      <c r="M74" s="9" t="n"/>
-      <c r="N74" s="9" t="n"/>
+      <c r="K74" s="9" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="4" t="n">
@@ -2491,16 +1814,7 @@
       <c r="H75" s="5" t="n"/>
       <c r="I75" s="6" t="n"/>
       <c r="J75" s="5" t="n"/>
-      <c r="K75" s="7">
-        <f>IF(J75&gt;0,G75/J75,0)</f>
-        <v/>
-      </c>
-      <c r="L75" s="7">
-        <f>MAX(G75-K75*(YEAR(TODAY())-YEAR(F75)),0)</f>
-        <v/>
-      </c>
-      <c r="M75" s="5" t="n"/>
-      <c r="N75" s="5" t="n"/>
+      <c r="K75" s="5" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="8" t="n">
@@ -2515,16 +1829,7 @@
       <c r="H76" s="9" t="n"/>
       <c r="I76" s="10" t="n"/>
       <c r="J76" s="9" t="n"/>
-      <c r="K76" s="11">
-        <f>IF(J76&gt;0,G76/J76,0)</f>
-        <v/>
-      </c>
-      <c r="L76" s="11">
-        <f>MAX(G76-K76*(YEAR(TODAY())-YEAR(F76)),0)</f>
-        <v/>
-      </c>
-      <c r="M76" s="9" t="n"/>
-      <c r="N76" s="9" t="n"/>
+      <c r="K76" s="9" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="4" t="n">
@@ -2539,16 +1844,7 @@
       <c r="H77" s="5" t="n"/>
       <c r="I77" s="6" t="n"/>
       <c r="J77" s="5" t="n"/>
-      <c r="K77" s="7">
-        <f>IF(J77&gt;0,G77/J77,0)</f>
-        <v/>
-      </c>
-      <c r="L77" s="7">
-        <f>MAX(G77-K77*(YEAR(TODAY())-YEAR(F77)),0)</f>
-        <v/>
-      </c>
-      <c r="M77" s="5" t="n"/>
-      <c r="N77" s="5" t="n"/>
+      <c r="K77" s="5" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="8" t="n">
@@ -2563,16 +1859,7 @@
       <c r="H78" s="9" t="n"/>
       <c r="I78" s="10" t="n"/>
       <c r="J78" s="9" t="n"/>
-      <c r="K78" s="11">
-        <f>IF(J78&gt;0,G78/J78,0)</f>
-        <v/>
-      </c>
-      <c r="L78" s="11">
-        <f>MAX(G78-K78*(YEAR(TODAY())-YEAR(F78)),0)</f>
-        <v/>
-      </c>
-      <c r="M78" s="9" t="n"/>
-      <c r="N78" s="9" t="n"/>
+      <c r="K78" s="9" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="4" t="n">
@@ -2587,16 +1874,7 @@
       <c r="H79" s="5" t="n"/>
       <c r="I79" s="6" t="n"/>
       <c r="J79" s="5" t="n"/>
-      <c r="K79" s="7">
-        <f>IF(J79&gt;0,G79/J79,0)</f>
-        <v/>
-      </c>
-      <c r="L79" s="7">
-        <f>MAX(G79-K79*(YEAR(TODAY())-YEAR(F79)),0)</f>
-        <v/>
-      </c>
-      <c r="M79" s="5" t="n"/>
-      <c r="N79" s="5" t="n"/>
+      <c r="K79" s="5" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="8" t="n">
@@ -2611,16 +1889,7 @@
       <c r="H80" s="9" t="n"/>
       <c r="I80" s="10" t="n"/>
       <c r="J80" s="9" t="n"/>
-      <c r="K80" s="11">
-        <f>IF(J80&gt;0,G80/J80,0)</f>
-        <v/>
-      </c>
-      <c r="L80" s="11">
-        <f>MAX(G80-K80*(YEAR(TODAY())-YEAR(F80)),0)</f>
-        <v/>
-      </c>
-      <c r="M80" s="9" t="n"/>
-      <c r="N80" s="9" t="n"/>
+      <c r="K80" s="9" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="4" t="n">
@@ -2635,16 +1904,7 @@
       <c r="H81" s="5" t="n"/>
       <c r="I81" s="6" t="n"/>
       <c r="J81" s="5" t="n"/>
-      <c r="K81" s="7">
-        <f>IF(J81&gt;0,G81/J81,0)</f>
-        <v/>
-      </c>
-      <c r="L81" s="7">
-        <f>MAX(G81-K81*(YEAR(TODAY())-YEAR(F81)),0)</f>
-        <v/>
-      </c>
-      <c r="M81" s="5" t="n"/>
-      <c r="N81" s="5" t="n"/>
+      <c r="K81" s="5" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="8" t="n">
@@ -2659,16 +1919,7 @@
       <c r="H82" s="9" t="n"/>
       <c r="I82" s="10" t="n"/>
       <c r="J82" s="9" t="n"/>
-      <c r="K82" s="11">
-        <f>IF(J82&gt;0,G82/J82,0)</f>
-        <v/>
-      </c>
-      <c r="L82" s="11">
-        <f>MAX(G82-K82*(YEAR(TODAY())-YEAR(F82)),0)</f>
-        <v/>
-      </c>
-      <c r="M82" s="9" t="n"/>
-      <c r="N82" s="9" t="n"/>
+      <c r="K82" s="9" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="4" t="n">
@@ -2683,16 +1934,7 @@
       <c r="H83" s="5" t="n"/>
       <c r="I83" s="6" t="n"/>
       <c r="J83" s="5" t="n"/>
-      <c r="K83" s="7">
-        <f>IF(J83&gt;0,G83/J83,0)</f>
-        <v/>
-      </c>
-      <c r="L83" s="7">
-        <f>MAX(G83-K83*(YEAR(TODAY())-YEAR(F83)),0)</f>
-        <v/>
-      </c>
-      <c r="M83" s="5" t="n"/>
-      <c r="N83" s="5" t="n"/>
+      <c r="K83" s="5" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="8" t="n">
@@ -2707,16 +1949,7 @@
       <c r="H84" s="9" t="n"/>
       <c r="I84" s="10" t="n"/>
       <c r="J84" s="9" t="n"/>
-      <c r="K84" s="11">
-        <f>IF(J84&gt;0,G84/J84,0)</f>
-        <v/>
-      </c>
-      <c r="L84" s="11">
-        <f>MAX(G84-K84*(YEAR(TODAY())-YEAR(F84)),0)</f>
-        <v/>
-      </c>
-      <c r="M84" s="9" t="n"/>
-      <c r="N84" s="9" t="n"/>
+      <c r="K84" s="9" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="4" t="n">
@@ -2731,16 +1964,7 @@
       <c r="H85" s="5" t="n"/>
       <c r="I85" s="6" t="n"/>
       <c r="J85" s="5" t="n"/>
-      <c r="K85" s="7">
-        <f>IF(J85&gt;0,G85/J85,0)</f>
-        <v/>
-      </c>
-      <c r="L85" s="7">
-        <f>MAX(G85-K85*(YEAR(TODAY())-YEAR(F85)),0)</f>
-        <v/>
-      </c>
-      <c r="M85" s="5" t="n"/>
-      <c r="N85" s="5" t="n"/>
+      <c r="K85" s="5" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="8" t="n">
@@ -2755,16 +1979,7 @@
       <c r="H86" s="9" t="n"/>
       <c r="I86" s="10" t="n"/>
       <c r="J86" s="9" t="n"/>
-      <c r="K86" s="11">
-        <f>IF(J86&gt;0,G86/J86,0)</f>
-        <v/>
-      </c>
-      <c r="L86" s="11">
-        <f>MAX(G86-K86*(YEAR(TODAY())-YEAR(F86)),0)</f>
-        <v/>
-      </c>
-      <c r="M86" s="9" t="n"/>
-      <c r="N86" s="9" t="n"/>
+      <c r="K86" s="9" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="4" t="n">
@@ -2779,16 +1994,7 @@
       <c r="H87" s="5" t="n"/>
       <c r="I87" s="6" t="n"/>
       <c r="J87" s="5" t="n"/>
-      <c r="K87" s="7">
-        <f>IF(J87&gt;0,G87/J87,0)</f>
-        <v/>
-      </c>
-      <c r="L87" s="7">
-        <f>MAX(G87-K87*(YEAR(TODAY())-YEAR(F87)),0)</f>
-        <v/>
-      </c>
-      <c r="M87" s="5" t="n"/>
-      <c r="N87" s="5" t="n"/>
+      <c r="K87" s="5" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="8" t="n">
@@ -2803,16 +2009,7 @@
       <c r="H88" s="9" t="n"/>
       <c r="I88" s="10" t="n"/>
       <c r="J88" s="9" t="n"/>
-      <c r="K88" s="11">
-        <f>IF(J88&gt;0,G88/J88,0)</f>
-        <v/>
-      </c>
-      <c r="L88" s="11">
-        <f>MAX(G88-K88*(YEAR(TODAY())-YEAR(F88)),0)</f>
-        <v/>
-      </c>
-      <c r="M88" s="9" t="n"/>
-      <c r="N88" s="9" t="n"/>
+      <c r="K88" s="9" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="4" t="n">
@@ -2827,16 +2024,7 @@
       <c r="H89" s="5" t="n"/>
       <c r="I89" s="6" t="n"/>
       <c r="J89" s="5" t="n"/>
-      <c r="K89" s="7">
-        <f>IF(J89&gt;0,G89/J89,0)</f>
-        <v/>
-      </c>
-      <c r="L89" s="7">
-        <f>MAX(G89-K89*(YEAR(TODAY())-YEAR(F89)),0)</f>
-        <v/>
-      </c>
-      <c r="M89" s="5" t="n"/>
-      <c r="N89" s="5" t="n"/>
+      <c r="K89" s="5" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="8" t="n">
@@ -2851,16 +2039,7 @@
       <c r="H90" s="9" t="n"/>
       <c r="I90" s="10" t="n"/>
       <c r="J90" s="9" t="n"/>
-      <c r="K90" s="11">
-        <f>IF(J90&gt;0,G90/J90,0)</f>
-        <v/>
-      </c>
-      <c r="L90" s="11">
-        <f>MAX(G90-K90*(YEAR(TODAY())-YEAR(F90)),0)</f>
-        <v/>
-      </c>
-      <c r="M90" s="9" t="n"/>
-      <c r="N90" s="9" t="n"/>
+      <c r="K90" s="9" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="4" t="n">
@@ -2875,16 +2054,7 @@
       <c r="H91" s="5" t="n"/>
       <c r="I91" s="6" t="n"/>
       <c r="J91" s="5" t="n"/>
-      <c r="K91" s="7">
-        <f>IF(J91&gt;0,G91/J91,0)</f>
-        <v/>
-      </c>
-      <c r="L91" s="7">
-        <f>MAX(G91-K91*(YEAR(TODAY())-YEAR(F91)),0)</f>
-        <v/>
-      </c>
-      <c r="M91" s="5" t="n"/>
-      <c r="N91" s="5" t="n"/>
+      <c r="K91" s="5" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="8" t="n">
@@ -2899,16 +2069,7 @@
       <c r="H92" s="9" t="n"/>
       <c r="I92" s="10" t="n"/>
       <c r="J92" s="9" t="n"/>
-      <c r="K92" s="11">
-        <f>IF(J92&gt;0,G92/J92,0)</f>
-        <v/>
-      </c>
-      <c r="L92" s="11">
-        <f>MAX(G92-K92*(YEAR(TODAY())-YEAR(F92)),0)</f>
-        <v/>
-      </c>
-      <c r="M92" s="9" t="n"/>
-      <c r="N92" s="9" t="n"/>
+      <c r="K92" s="9" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="4" t="n">
@@ -2923,16 +2084,7 @@
       <c r="H93" s="5" t="n"/>
       <c r="I93" s="6" t="n"/>
       <c r="J93" s="5" t="n"/>
-      <c r="K93" s="7">
-        <f>IF(J93&gt;0,G93/J93,0)</f>
-        <v/>
-      </c>
-      <c r="L93" s="7">
-        <f>MAX(G93-K93*(YEAR(TODAY())-YEAR(F93)),0)</f>
-        <v/>
-      </c>
-      <c r="M93" s="5" t="n"/>
-      <c r="N93" s="5" t="n"/>
+      <c r="K93" s="5" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="8" t="n">
@@ -2947,16 +2099,7 @@
       <c r="H94" s="9" t="n"/>
       <c r="I94" s="10" t="n"/>
       <c r="J94" s="9" t="n"/>
-      <c r="K94" s="11">
-        <f>IF(J94&gt;0,G94/J94,0)</f>
-        <v/>
-      </c>
-      <c r="L94" s="11">
-        <f>MAX(G94-K94*(YEAR(TODAY())-YEAR(F94)),0)</f>
-        <v/>
-      </c>
-      <c r="M94" s="9" t="n"/>
-      <c r="N94" s="9" t="n"/>
+      <c r="K94" s="9" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="4" t="n">
@@ -2971,16 +2114,7 @@
       <c r="H95" s="5" t="n"/>
       <c r="I95" s="6" t="n"/>
       <c r="J95" s="5" t="n"/>
-      <c r="K95" s="7">
-        <f>IF(J95&gt;0,G95/J95,0)</f>
-        <v/>
-      </c>
-      <c r="L95" s="7">
-        <f>MAX(G95-K95*(YEAR(TODAY())-YEAR(F95)),0)</f>
-        <v/>
-      </c>
-      <c r="M95" s="5" t="n"/>
-      <c r="N95" s="5" t="n"/>
+      <c r="K95" s="5" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="8" t="n">
@@ -2995,16 +2129,7 @@
       <c r="H96" s="9" t="n"/>
       <c r="I96" s="10" t="n"/>
       <c r="J96" s="9" t="n"/>
-      <c r="K96" s="11">
-        <f>IF(J96&gt;0,G96/J96,0)</f>
-        <v/>
-      </c>
-      <c r="L96" s="11">
-        <f>MAX(G96-K96*(YEAR(TODAY())-YEAR(F96)),0)</f>
-        <v/>
-      </c>
-      <c r="M96" s="9" t="n"/>
-      <c r="N96" s="9" t="n"/>
+      <c r="K96" s="9" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="4" t="n">
@@ -3019,16 +2144,7 @@
       <c r="H97" s="5" t="n"/>
       <c r="I97" s="6" t="n"/>
       <c r="J97" s="5" t="n"/>
-      <c r="K97" s="7">
-        <f>IF(J97&gt;0,G97/J97,0)</f>
-        <v/>
-      </c>
-      <c r="L97" s="7">
-        <f>MAX(G97-K97*(YEAR(TODAY())-YEAR(F97)),0)</f>
-        <v/>
-      </c>
-      <c r="M97" s="5" t="n"/>
-      <c r="N97" s="5" t="n"/>
+      <c r="K97" s="5" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="8" t="n">
@@ -3043,16 +2159,7 @@
       <c r="H98" s="9" t="n"/>
       <c r="I98" s="10" t="n"/>
       <c r="J98" s="9" t="n"/>
-      <c r="K98" s="11">
-        <f>IF(J98&gt;0,G98/J98,0)</f>
-        <v/>
-      </c>
-      <c r="L98" s="11">
-        <f>MAX(G98-K98*(YEAR(TODAY())-YEAR(F98)),0)</f>
-        <v/>
-      </c>
-      <c r="M98" s="9" t="n"/>
-      <c r="N98" s="9" t="n"/>
+      <c r="K98" s="9" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="4" t="n">
@@ -3067,16 +2174,7 @@
       <c r="H99" s="5" t="n"/>
       <c r="I99" s="6" t="n"/>
       <c r="J99" s="5" t="n"/>
-      <c r="K99" s="7">
-        <f>IF(J99&gt;0,G99/J99,0)</f>
-        <v/>
-      </c>
-      <c r="L99" s="7">
-        <f>MAX(G99-K99*(YEAR(TODAY())-YEAR(F99)),0)</f>
-        <v/>
-      </c>
-      <c r="M99" s="5" t="n"/>
-      <c r="N99" s="5" t="n"/>
+      <c r="K99" s="5" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="8" t="n">
@@ -3091,16 +2189,7 @@
       <c r="H100" s="9" t="n"/>
       <c r="I100" s="10" t="n"/>
       <c r="J100" s="9" t="n"/>
-      <c r="K100" s="11">
-        <f>IF(J100&gt;0,G100/J100,0)</f>
-        <v/>
-      </c>
-      <c r="L100" s="11">
-        <f>MAX(G100-K100*(YEAR(TODAY())-YEAR(F100)),0)</f>
-        <v/>
-      </c>
-      <c r="M100" s="9" t="n"/>
-      <c r="N100" s="9" t="n"/>
+      <c r="K100" s="9" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="4" t="n">
@@ -3115,16 +2204,7 @@
       <c r="H101" s="5" t="n"/>
       <c r="I101" s="6" t="n"/>
       <c r="J101" s="5" t="n"/>
-      <c r="K101" s="7">
-        <f>IF(J101&gt;0,G101/J101,0)</f>
-        <v/>
-      </c>
-      <c r="L101" s="7">
-        <f>MAX(G101-K101*(YEAR(TODAY())-YEAR(F101)),0)</f>
-        <v/>
-      </c>
-      <c r="M101" s="5" t="n"/>
-      <c r="N101" s="5" t="n"/>
+      <c r="K101" s="5" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="8" t="n">
@@ -3139,16 +2219,7 @@
       <c r="H102" s="9" t="n"/>
       <c r="I102" s="10" t="n"/>
       <c r="J102" s="9" t="n"/>
-      <c r="K102" s="11">
-        <f>IF(J102&gt;0,G102/J102,0)</f>
-        <v/>
-      </c>
-      <c r="L102" s="11">
-        <f>MAX(G102-K102*(YEAR(TODAY())-YEAR(F102)),0)</f>
-        <v/>
-      </c>
-      <c r="M102" s="9" t="n"/>
-      <c r="N102" s="9" t="n"/>
+      <c r="K102" s="9" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="12" t="inlineStr">
@@ -3168,20 +2239,11 @@
       <c r="H103" s="13" t="n"/>
       <c r="I103" s="13" t="n"/>
       <c r="J103" s="13" t="n"/>
-      <c r="K103" s="14">
-        <f>SUM(K3:K102)</f>
-        <v/>
-      </c>
-      <c r="L103" s="14">
-        <f>SUM(L3:L102)</f>
-        <v/>
-      </c>
-      <c r="M103" s="13" t="n"/>
-      <c r="N103" s="13" t="n"/>
+      <c r="K103" s="13" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <conditionalFormatting sqref="H3:H102">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
@@ -3207,7 +2269,7 @@
     <dataValidation sqref="H3 H4 H5 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34 H35 H36 H37 H38 H39 H40 H41 H42 H43 H44 H45 H46 H47 H48 H49 H50 H51 H52 H53 H54 H55 H56 H57 H58 H59 H60 H61 H62 H63 H64 H65 H66 H67 H68 H69 H70 H71 H72 H73 H74 H75 H76 H77 H78 H79 H80 H81 H82 H83 H84 H85 H86 H87 H88 H89 H90 H91 H92 H93 H94 H95 H96 H97 H98 H99 H100 H101 H102" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"New,Excellent,Good,Fair,Poor,Retired"</formula1>
     </dataValidation>
-    <dataValidation sqref="M3 M4 M5 M6 M7 M8 M9 M10 M11 M12 M13 M14 M15 M16 M17 M18 M19 M20 M21 M22 M23 M24 M25 M26 M27 M28 M29 M30 M31 M32 M33 M34 M35 M36 M37 M38 M39 M40 M41 M42 M43 M44 M45 M46 M47 M48 M49 M50 M51 M52 M53 M54 M55 M56 M57 M58 M59 M60 M61 M62 M63 M64 M65 M66 M67 M68 M69 M70 M71 M72 M73 M74 M75 M76 M77 M78 M79 M80 M81 M82 M83 M84 M85 M86 M87 M88 M89 M90 M91 M92 M93 M94 M95 M96 M97 M98 M99 M100 M101 M102" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J3 J4 J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J33 J34 J35 J36 J37 J38 J39 J40 J41 J42 J43 J44 J45 J46 J47 J48 J49 J50 J51 J52 J53 J54 J55 J56 J57 J58 J59 J60 J61 J62 J63 J64 J65 J66 J67 J68 J69 J70 J71 J72 J73 J74 J75 J76 J77 J78 J79 J80 J81 J82 J83 J84 J85 J86 J87 J88 J89 J90 J91 J92 J93 J94 J95 J96 J97 J98 J99 J100 J101 J102" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Truck,Garage,Job Site,Storage,Office"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat: add 8 equipment items with correct brand/model details
STIHL FS 40 C-E, Husqvarna 150BT backpack blower (renewed),
Trailer 5X8, electric blower, Ariens riding mower, Echo SRM-2620AA
X Series, Greenworks 40V dethatcher/scarifier, Proyama 24in hedger.
12 total assets pre-populated.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TotalGuard_2026_Equipment_Inventory.xlsx
+++ b/TotalGuard_2026_Equipment_Inventory.xlsx
@@ -785,121 +785,293 @@
       <c r="A7" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B7" s="5" t="n"/>
-      <c r="C7" s="5" t="n"/>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="5" t="n"/>
-      <c r="F7" s="6" t="n"/>
-      <c r="G7" s="7" t="n"/>
-      <c r="H7" s="5" t="n"/>
-      <c r="I7" s="6" t="n"/>
-      <c r="J7" s="5" t="n"/>
-      <c r="K7" s="5" t="n"/>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>STIHL String Trimmer</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Trimmer</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>STIHL FS 40 C-E Gas</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="6" t="inlineStr"/>
+      <c r="G7" s="7" t="n">
+        <v>200</v>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="inlineStr"/>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>Truck</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="9" t="n"/>
-      <c r="C8" s="9" t="n"/>
-      <c r="D8" s="9" t="n"/>
-      <c r="E8" s="9" t="n"/>
-      <c r="F8" s="10" t="n"/>
-      <c r="G8" s="11" t="n"/>
-      <c r="H8" s="9" t="n"/>
-      <c r="I8" s="10" t="n"/>
-      <c r="J8" s="9" t="n"/>
-      <c r="K8" s="9" t="n"/>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Husqvarna Backpack Blower</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Blower</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>Husqvarna 150BT 952991658 50.2cc 270mph</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr"/>
+      <c r="F8" s="10" t="inlineStr"/>
+      <c r="G8" s="11" t="n">
+        <v>200</v>
+      </c>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="I8" s="10" t="inlineStr"/>
+      <c r="J8" s="9" t="inlineStr">
+        <is>
+          <t>Truck</t>
+        </is>
+      </c>
+      <c r="K8" s="9" t="inlineStr">
+        <is>
+          <t>Renewed from Amazon</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="B9" s="5" t="n"/>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="5" t="n"/>
-      <c r="F9" s="6" t="n"/>
-      <c r="G9" s="7" t="n"/>
-      <c r="H9" s="5" t="n"/>
-      <c r="I9" s="6" t="n"/>
-      <c r="J9" s="5" t="n"/>
-      <c r="K9" s="5" t="n"/>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Trailer 5X8</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Trailer</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr"/>
+      <c r="E9" s="5" t="inlineStr"/>
+      <c r="F9" s="6" t="inlineStr"/>
+      <c r="G9" s="7" t="n">
+        <v>400</v>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="inlineStr"/>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>Truck</t>
+        </is>
+      </c>
+      <c r="K9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="B10" s="9" t="n"/>
-      <c r="C10" s="9" t="n"/>
-      <c r="D10" s="9" t="n"/>
-      <c r="E10" s="9" t="n"/>
-      <c r="F10" s="10" t="n"/>
-      <c r="G10" s="11" t="n"/>
-      <c r="H10" s="9" t="n"/>
-      <c r="I10" s="10" t="n"/>
-      <c r="J10" s="9" t="n"/>
-      <c r="K10" s="9" t="n"/>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Electric Blower</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>Blower</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr"/>
+      <c r="E10" s="9" t="inlineStr"/>
+      <c r="F10" s="10" t="inlineStr"/>
+      <c r="G10" s="11" t="n">
+        <v>200</v>
+      </c>
+      <c r="H10" s="9" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="I10" s="10" t="inlineStr"/>
+      <c r="J10" s="9" t="inlineStr">
+        <is>
+          <t>Truck</t>
+        </is>
+      </c>
+      <c r="K10" s="9" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="B11" s="5" t="n"/>
-      <c r="C11" s="5" t="n"/>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="5" t="n"/>
-      <c r="F11" s="6" t="n"/>
-      <c r="G11" s="7" t="n"/>
-      <c r="H11" s="5" t="n"/>
-      <c r="I11" s="6" t="n"/>
-      <c r="J11" s="5" t="n"/>
-      <c r="K11" s="5" t="n"/>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Ariens Riding Mower</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Mower</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Ariens</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr"/>
+      <c r="F11" s="6" t="inlineStr"/>
+      <c r="G11" s="7" t="n">
+        <v>3956</v>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr"/>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>Garage</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="8" t="n">
         <v>10</v>
       </c>
-      <c r="B12" s="9" t="n"/>
-      <c r="C12" s="9" t="n"/>
-      <c r="D12" s="9" t="n"/>
-      <c r="E12" s="9" t="n"/>
-      <c r="F12" s="10" t="n"/>
-      <c r="G12" s="11" t="n"/>
-      <c r="H12" s="9" t="n"/>
-      <c r="I12" s="10" t="n"/>
-      <c r="J12" s="9" t="n"/>
-      <c r="K12" s="9" t="n"/>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Echo String Trimmer</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>Trimmer</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Echo SRM-2620AA 25.4cc X Series Straight Shaft</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr"/>
+      <c r="F12" s="10" t="inlineStr"/>
+      <c r="G12" s="11" t="n">
+        <v>399</v>
+      </c>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="I12" s="10" t="inlineStr"/>
+      <c r="J12" s="9" t="inlineStr">
+        <is>
+          <t>Truck</t>
+        </is>
+      </c>
+      <c r="K12" s="9" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="B13" s="5" t="n"/>
-      <c r="C13" s="5" t="n"/>
-      <c r="D13" s="5" t="n"/>
-      <c r="E13" s="5" t="n"/>
-      <c r="F13" s="6" t="n"/>
-      <c r="G13" s="7" t="n"/>
-      <c r="H13" s="5" t="n"/>
-      <c r="I13" s="6" t="n"/>
-      <c r="J13" s="5" t="n"/>
-      <c r="K13" s="5" t="n"/>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Greenworks Dethatcher/Scarifier</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Aerator</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Greenworks 40V 15in</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr"/>
+      <c r="F13" s="6" t="inlineStr"/>
+      <c r="G13" s="7" t="n">
+        <v>249.99</v>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="inlineStr"/>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>Garage</t>
+        </is>
+      </c>
+      <c r="K13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="8" t="n">
         <v>12</v>
       </c>
-      <c r="B14" s="9" t="n"/>
-      <c r="C14" s="9" t="n"/>
-      <c r="D14" s="9" t="n"/>
-      <c r="E14" s="9" t="n"/>
-      <c r="F14" s="10" t="n"/>
-      <c r="G14" s="11" t="n"/>
-      <c r="H14" s="9" t="n"/>
-      <c r="I14" s="10" t="n"/>
-      <c r="J14" s="9" t="n"/>
-      <c r="K14" s="9" t="n"/>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Proyama Dual Sided Hedger</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>Trimmer</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>Proyama 24in 26cc 2-Cycle Gas</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr"/>
+      <c r="F14" s="10" t="inlineStr"/>
+      <c r="G14" s="11" t="n">
+        <v>179</v>
+      </c>
+      <c r="H14" s="9" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="I14" s="10" t="inlineStr"/>
+      <c r="J14" s="9" t="inlineStr">
+        <is>
+          <t>Truck</t>
+        </is>
+      </c>
+      <c r="K14" s="9" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">

</xml_diff>